<commit_message>
Some changes during the course
</commit_message>
<xml_diff>
--- a/New design.xlsx
+++ b/New design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\2025 Scotlan Level 8 courses\Mod-4 Implementing Software\New course by Mike\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\2025 Scotland Level 8 courses\Mod-4 Implementing Software\New course by Mike\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A8C4359E-0B2D-440B-8622-19F83A137525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFF973E-9310-4DA3-A0CC-EE6EC8874029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{9055093E-C582-4D7E-A85B-4A6CC7DA55DA}"/>
+    <workbookView xWindow="5484" yWindow="2328" windowWidth="17280" windowHeight="17220" xr2:uid="{9055093E-C582-4D7E-A85B-4A6CC7DA55DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
   <si>
     <t>Morning</t>
   </si>
@@ -481,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A73B5E2-127B-4046-B556-DD223C5A52C6}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
@@ -646,6 +646,11 @@
       </c>
       <c r="E13" s="2"/>
     </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added the intro slide
</commit_message>
<xml_diff>
--- a/New design.xlsx
+++ b/New design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\2025 Scotland Level 8 courses\Mod-4 Implementing Software\New course by Mike\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\Scotland\2025 Scotland Level 8 courses\Mod-4 Implementing Software\New course by Mike\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AFF973E-9310-4DA3-A0CC-EE6EC8874029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83179B51-9B4A-4111-8A41-BC411F59EBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5484" yWindow="2328" windowWidth="17280" windowHeight="17220" xr2:uid="{9055093E-C582-4D7E-A85B-4A6CC7DA55DA}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{9055093E-C582-4D7E-A85B-4A6CC7DA55DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
   <si>
     <t>Morning</t>
   </si>
@@ -93,6 +93,12 @@
   </si>
   <si>
     <t>total</t>
+  </si>
+  <si>
+    <t>No need for UML, ERD</t>
+  </si>
+  <si>
+    <t>Needs to include GIT, Deploytment, Branching, Merging, Jira</t>
   </si>
 </sst>
 </file>
@@ -481,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A73B5E2-127B-4046-B556-DD223C5A52C6}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
@@ -489,7 +495,7 @@
     <col min="5" max="5" width="4.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
         <v>8</v>
@@ -498,7 +504,7 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" t="s">
         <v>13</v>
@@ -511,7 +517,7 @@
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" t="s">
         <v>13</v>
@@ -524,7 +530,7 @@
       </c>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" t="s">
         <v>0</v>
@@ -536,8 +542,11 @@
         <v>2</v>
       </c>
       <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="1" t="s">
         <v>4</v>
@@ -549,8 +558,11 @@
         <v>2</v>
       </c>
       <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" t="s">
         <v>5</v>
@@ -563,7 +575,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" t="s">
         <v>5</v>
@@ -576,7 +588,7 @@
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
@@ -587,7 +599,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
         <v>9</v>
@@ -596,7 +608,7 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" t="s">
         <v>0</v>
@@ -609,7 +621,7 @@
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="1" t="s">
         <v>4</v>
@@ -622,7 +634,7 @@
       </c>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" t="s">
         <v>5</v>
@@ -635,7 +647,7 @@
       </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
@@ -646,7 +658,7 @@
       </c>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>5</v>
       </c>

</xml_diff>